<commit_message>
Add change 2023-2025 view to STR summary (YoY % + yearly line charts)
- Overview tab: %Chg columns (STR's own YoY + computed 25v23) and a yearly
  line chart per metric
- HTML report: Change 2023-2025 section with yearly mini charts and arrows

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzrfbzxdPZVRCw2bYpGG1J
</commit_message>
<xml_diff>
--- a/output/STR_Bangkok_by_segment_2023-2025.xlsx
+++ b/output/STR_Bangkok_by_segment_2023-2025.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="+0.0&quot;%&quot;;-0.0&quot;%&quot;;0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +54,12 @@
     <font>
       <b val="1"/>
       <color rgb="002A78D6"/>
+    </font>
+    <font>
+      <color rgb="00006300"/>
+    </font>
+    <font>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -111,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,13 +131,19 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -210,6 +223,708 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Occupancy (%) — yearly average</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$6:$D$6</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$7:$D$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EDA100"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$8:$D$8</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$D$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$9:$D$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>ADR (THB) — yearly average</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A21</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$22:$D$22</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A23</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$23:$D$23</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A24</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EDA100"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$24:$D$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$D$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$25:$D$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>RevPAR (THB) — yearly average</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A37</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$38:$D$38</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$39:$D$39</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A40</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="EDA100"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$40:$D$40</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$D$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$41:$D$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
@@ -441,7 +1156,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -674,7 +1389,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -911,12 +1626,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9360000" cy="3420000"/>
+    <ext cx="4860000" cy="2592000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -926,6 +1641,50 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4860000" cy="2592000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4860000" cy="2592000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -962,6 +1721,33 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1277,26 +2063,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bangkok STR — market class comparison</t>
+          <t>Bangkok STR — market class comparison: change 2023–2025</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yearly averages by market class (STR 'Total' rows). Occupancy = %, ADR &amp; RevPAR = THB.</t>
+          <t>Yearly averages by market class (STR 'Total' rows) with % change. Occupancy = %, ADR &amp; RevPAR = THB. '24 vs 23' / '25 vs 24' are STR's own % Chg.</t>
         </is>
       </c>
     </row>
@@ -1328,6 +2117,21 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>24 vs 23</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 24</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 23</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1344,9 +2148,18 @@
       <c r="D6" s="7" t="n">
         <v>67</v>
       </c>
+      <c r="E6" s="8" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>-8.699999999999999</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>-2.5</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Upper Upscale</t>
         </is>
@@ -1360,9 +2173,18 @@
       <c r="D7" s="7" t="n">
         <v>69.59999999999999</v>
       </c>
+      <c r="E7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>-3.5</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Upscale</t>
         </is>
@@ -1376,9 +2198,18 @@
       <c r="D8" s="7" t="n">
         <v>74.2</v>
       </c>
+      <c r="E8" s="8" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>3.9</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Upper Midscale</t>
         </is>
@@ -1392,195 +2223,307 @@
       <c r="D9" s="7" t="n">
         <v>75.90000000000001</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="E9" s="8" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>ADR (THB)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Market class</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>24 vs 23</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 24</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Luxury</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B22" s="13" t="n">
         <v>6685</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C22" s="13" t="n">
         <v>6984</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D22" s="13" t="n">
         <v>6998</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Upper Upscale</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n">
-        <v>4258</v>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>4492</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>4391</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Upscale</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="n">
-        <v>2906</v>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>3148</v>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>3099</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Upper Midscale</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n">
-        <v>2548</v>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>2831</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>2813</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>RevPAR (THB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Market class</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Luxury</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="n">
-        <v>4593</v>
-      </c>
-      <c r="C20" s="11" t="n">
-        <v>5129</v>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>4691</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Upper Upscale</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="n">
-        <v>3073</v>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>3405</v>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>3057</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>Upscale</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="n">
-        <v>2073</v>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>2423</v>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>2298</v>
+      <c r="E22" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>4.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
+          <t>Upper Upscale</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>4258</v>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>4492</v>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>4391</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Upscale</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>2906</v>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>3148</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>3099</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
           <t>Upper Midscale</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B25" s="13" t="n">
+        <v>2548</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>2831</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>2813</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>RevPAR (THB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Market class</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>24 vs 23</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 24</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>25 vs 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>4593</v>
+      </c>
+      <c r="C38" s="13" t="n">
+        <v>5129</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>4691</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Upper Upscale</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="n">
+        <v>3073</v>
+      </c>
+      <c r="C39" s="13" t="n">
+        <v>3405</v>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>3057</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>-10.2</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Upscale</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="n">
+        <v>2073</v>
+      </c>
+      <c r="C40" s="13" t="n">
+        <v>2423</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>2298</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Upper Midscale</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
         <v>1827</v>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C41" s="13" t="n">
         <v>2161</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D41" s="13" t="n">
         <v>2135</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <v>16.8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1601,7 +2544,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Bangkok STR — Occupancy by market class (monthly, This Year)</t>
         </is>
@@ -1642,7 +2585,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
@@ -1661,7 +2604,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
@@ -1680,7 +2623,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
@@ -1699,7 +2642,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
@@ -1718,7 +2661,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
@@ -1737,7 +2680,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
@@ -1756,7 +2699,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
@@ -1775,7 +2718,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
@@ -1794,7 +2737,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
@@ -1813,7 +2756,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
@@ -1832,7 +2775,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
@@ -1851,7 +2794,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
@@ -1870,7 +2813,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
@@ -1889,7 +2832,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
@@ -1908,7 +2851,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
@@ -1927,7 +2870,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
@@ -1946,7 +2889,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
@@ -1965,7 +2908,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
@@ -1984,7 +2927,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
@@ -2003,7 +2946,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
@@ -2022,7 +2965,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
@@ -2041,7 +2984,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
@@ -2060,7 +3003,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
@@ -2079,7 +3022,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
@@ -2098,7 +3041,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
@@ -2117,7 +3060,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -2136,7 +3079,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
@@ -2155,7 +3098,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
@@ -2174,7 +3117,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
@@ -2193,7 +3136,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
@@ -2212,7 +3155,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
@@ -2231,7 +3174,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
@@ -2250,7 +3193,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
@@ -2269,7 +3212,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
@@ -2288,7 +3231,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
@@ -2307,7 +3250,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
@@ -2348,7 +3291,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Bangkok STR — ADR by market class (monthly, This Year)</t>
         </is>
@@ -2389,686 +3332,686 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="13" t="n">
         <v>7257.67</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="13" t="n">
         <v>4324.77</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="13" t="n">
         <v>2863.43</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="13" t="n">
         <v>2469.09</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="13" t="n">
         <v>6650.01</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="13" t="n">
         <v>4201.15</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="13" t="n">
         <v>2829.5</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="13" t="n">
         <v>2395.04</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="13" t="n">
         <v>6489.71</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="13" t="n">
         <v>4235.39</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="13" t="n">
         <v>2890.68</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <v>2443.81</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="13" t="n">
         <v>6949.89</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="13" t="n">
         <v>4309.86</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="13" t="n">
         <v>2879.78</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <v>2485.27</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="13" t="n">
         <v>6174.16</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="13" t="n">
         <v>4063.43</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="13" t="n">
         <v>2745.19</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="13" t="n">
         <v>2357.71</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="13" t="n">
         <v>6145.31</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="13" t="n">
         <v>4084.32</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="13" t="n">
         <v>2815.39</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="13" t="n">
         <v>2434.92</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="13" t="n">
         <v>6593.69</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="13" t="n">
         <v>4220.41</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="13" t="n">
         <v>2974.75</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="13" t="n">
         <v>2560.81</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
         <v>6499</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="13" t="n">
         <v>4222.3</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="13" t="n">
         <v>2937.66</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="13" t="n">
         <v>2612.55</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="13" t="n">
         <v>6004.24</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="13" t="n">
         <v>4003.59</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="13" t="n">
         <v>2747.58</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="13" t="n">
         <v>2515.08</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="13" t="n">
         <v>6310.62</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="13" t="n">
         <v>4070.44</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="13" t="n">
         <v>2760.38</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="13" t="n">
         <v>2482.23</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="13" t="n">
         <v>6636.91</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="13" t="n">
         <v>4332.99</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="13" t="n">
         <v>2984.16</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="13" t="n">
         <v>2682.9</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="13" t="n">
         <v>8183.87</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="13" t="n">
         <v>4906.12</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="13" t="n">
         <v>3341.61</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="13" t="n">
         <v>3038.37</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="13" t="n">
         <v>7232.85</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="13" t="n">
         <v>4449.88</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="13" t="n">
         <v>3027</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="13" t="n">
         <v>2695.29</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="13" t="n">
         <v>7511.89</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="13" t="n">
         <v>4711.27</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="13" t="n">
         <v>3259.63</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="13" t="n">
         <v>2876.63</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="13" t="n">
         <v>6678.36</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="13" t="n">
         <v>4349.05</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="13" t="n">
         <v>3000.15</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="13" t="n">
         <v>2661.83</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="13" t="n">
         <v>6807.84</v>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="13" t="n">
         <v>4374.91</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="13" t="n">
         <v>3020.58</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="13" t="n">
         <v>2684.7</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="13" t="n">
         <v>6383.14</v>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="13" t="n">
         <v>4216.76</v>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D21" s="13" t="n">
         <v>2910.82</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="13" t="n">
         <v>2589.48</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="13" t="n">
         <v>6435.11</v>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="13" t="n">
         <v>4256.48</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="13" t="n">
         <v>2996.93</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="13" t="n">
         <v>2667.56</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="13" t="n">
         <v>6765.18</v>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C23" s="13" t="n">
         <v>4405.22</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D23" s="13" t="n">
         <v>3138.3</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="13" t="n">
         <v>2803.39</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="13" t="n">
         <v>6914.04</v>
       </c>
-      <c r="C24" s="11" t="n">
+      <c r="C24" s="13" t="n">
         <v>4556.91</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="13" t="n">
         <v>3238.95</v>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="13" t="n">
         <v>2908.9</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B25" s="13" t="n">
         <v>6115.68</v>
       </c>
-      <c r="C25" s="11" t="n">
+      <c r="C25" s="13" t="n">
         <v>4132.36</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="13" t="n">
         <v>2912.96</v>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="13" t="n">
         <v>2673.8</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="13" t="n">
         <v>6438.59</v>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C26" s="13" t="n">
         <v>4174.16</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="13" t="n">
         <v>2938.5</v>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="13" t="n">
         <v>2709.8</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="13" t="n">
         <v>7230.78</v>
       </c>
-      <c r="C27" s="11" t="n">
+      <c r="C27" s="13" t="n">
         <v>4771.42</v>
       </c>
-      <c r="D27" s="11" t="n">
+      <c r="D27" s="13" t="n">
         <v>3413.37</v>
       </c>
-      <c r="E27" s="11" t="n">
+      <c r="E27" s="13" t="n">
         <v>3097.43</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="13" t="n">
         <v>8865.09</v>
       </c>
-      <c r="C28" s="11" t="n">
+      <c r="C28" s="13" t="n">
         <v>5305.73</v>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D28" s="13" t="n">
         <v>3776.59</v>
       </c>
-      <c r="E28" s="11" t="n">
+      <c r="E28" s="13" t="n">
         <v>3466.66</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B29" s="13" t="n">
         <v>8155.43</v>
       </c>
-      <c r="C29" s="11" t="n">
+      <c r="C29" s="13" t="n">
         <v>4881.25</v>
       </c>
-      <c r="D29" s="11" t="n">
+      <c r="D29" s="13" t="n">
         <v>3479.24</v>
       </c>
-      <c r="E29" s="11" t="n">
+      <c r="E29" s="13" t="n">
         <v>3216.07</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="13" t="n">
         <v>7324.96</v>
       </c>
-      <c r="C30" s="11" t="n">
+      <c r="C30" s="13" t="n">
         <v>4680.93</v>
       </c>
-      <c r="D30" s="11" t="n">
+      <c r="D30" s="13" t="n">
         <v>3329.91</v>
       </c>
-      <c r="E30" s="11" t="n">
+      <c r="E30" s="13" t="n">
         <v>3048.34</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n">
+      <c r="B31" s="13" t="n">
         <v>6728.43</v>
       </c>
-      <c r="C31" s="11" t="n">
+      <c r="C31" s="13" t="n">
         <v>4343.3</v>
       </c>
-      <c r="D31" s="11" t="n">
+      <c r="D31" s="13" t="n">
         <v>3091.87</v>
       </c>
-      <c r="E31" s="11" t="n">
+      <c r="E31" s="13" t="n">
         <v>2805.96</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="13" t="n">
         <v>6827.43</v>
       </c>
-      <c r="C32" s="11" t="n">
+      <c r="C32" s="13" t="n">
         <v>4265.86</v>
       </c>
-      <c r="D32" s="11" t="n">
+      <c r="D32" s="13" t="n">
         <v>3038.34</v>
       </c>
-      <c r="E32" s="11" t="n">
+      <c r="E32" s="13" t="n">
         <v>2694.61</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="13" t="n">
         <v>6332.58</v>
       </c>
-      <c r="C33" s="11" t="n">
+      <c r="C33" s="13" t="n">
         <v>4184.04</v>
       </c>
-      <c r="D33" s="11" t="n">
+      <c r="D33" s="13" t="n">
         <v>2877.48</v>
       </c>
-      <c r="E33" s="11" t="n">
+      <c r="E33" s="13" t="n">
         <v>2573.31</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="13" t="n">
         <v>6218.14</v>
       </c>
-      <c r="C34" s="11" t="n">
+      <c r="C34" s="13" t="n">
         <v>4068.12</v>
       </c>
-      <c r="D34" s="11" t="n">
+      <c r="D34" s="13" t="n">
         <v>2885.56</v>
       </c>
-      <c r="E34" s="11" t="n">
+      <c r="E34" s="13" t="n">
         <v>2576.24</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="13" t="n">
         <v>6563.5</v>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C35" s="13" t="n">
         <v>4170.97</v>
       </c>
-      <c r="D35" s="11" t="n">
+      <c r="D35" s="13" t="n">
         <v>3010.69</v>
       </c>
-      <c r="E35" s="11" t="n">
+      <c r="E35" s="13" t="n">
         <v>2707.91</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
       </c>
-      <c r="B36" s="11" t="n">
+      <c r="B36" s="13" t="n">
         <v>6631.46</v>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C36" s="13" t="n">
         <v>4168.19</v>
       </c>
-      <c r="D36" s="11" t="n">
+      <c r="D36" s="13" t="n">
         <v>3034.68</v>
       </c>
-      <c r="E36" s="11" t="n">
+      <c r="E36" s="13" t="n">
         <v>2758.53</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B37" s="13" t="n">
         <v>5950.24</v>
       </c>
-      <c r="C37" s="11" t="n">
+      <c r="C37" s="13" t="n">
         <v>3898.96</v>
       </c>
-      <c r="D37" s="11" t="n">
+      <c r="D37" s="13" t="n">
         <v>2773.08</v>
       </c>
-      <c r="E37" s="11" t="n">
+      <c r="E37" s="13" t="n">
         <v>2519.21</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B38" s="11" t="n">
+      <c r="B38" s="13" t="n">
         <v>6476.21</v>
       </c>
-      <c r="C38" s="11" t="n">
+      <c r="C38" s="13" t="n">
         <v>4096.54</v>
       </c>
-      <c r="D38" s="11" t="n">
+      <c r="D38" s="13" t="n">
         <v>2833.55</v>
       </c>
-      <c r="E38" s="11" t="n">
+      <c r="E38" s="13" t="n">
         <v>2628.42</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n">
+      <c r="B39" s="13" t="n">
         <v>6973.41</v>
       </c>
-      <c r="C39" s="11" t="n">
+      <c r="C39" s="13" t="n">
         <v>4483.61</v>
       </c>
-      <c r="D39" s="11" t="n">
+      <c r="D39" s="13" t="n">
         <v>3125.73</v>
       </c>
-      <c r="E39" s="11" t="n">
+      <c r="E39" s="13" t="n">
         <v>2849.07</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B40" s="11" t="n">
+      <c r="B40" s="13" t="n">
         <v>8911.91</v>
       </c>
-      <c r="C40" s="11" t="n">
+      <c r="C40" s="13" t="n">
         <v>5153.75</v>
       </c>
-      <c r="D40" s="11" t="n">
+      <c r="D40" s="13" t="n">
         <v>3562.61</v>
       </c>
-      <c r="E40" s="11" t="n">
+      <c r="E40" s="13" t="n">
         <v>3246.97</v>
       </c>
     </row>
@@ -3095,7 +4038,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Bangkok STR — RevPAR by market class (monthly, This Year)</t>
         </is>
@@ -3136,686 +4079,686 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="13" t="n">
         <v>4889.14</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="13" t="n">
         <v>2870.44</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="13" t="n">
         <v>1867.78</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="13" t="n">
         <v>1723.59</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="13" t="n">
         <v>4843.13</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="13" t="n">
         <v>3172.27</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="13" t="n">
         <v>2034.2</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="13" t="n">
         <v>1795.17</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="13" t="n">
         <v>4633.91</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="13" t="n">
         <v>3295.11</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="13" t="n">
         <v>2136.46</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <v>1811.98</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="13" t="n">
         <v>4641.89</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="13" t="n">
         <v>3093.95</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="13" t="n">
         <v>1960.92</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <v>1708.71</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="13" t="n">
         <v>3823.42</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="13" t="n">
         <v>2698.86</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="13" t="n">
         <v>1864.02</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="13" t="n">
         <v>1571.84</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="13" t="n">
         <v>3907.12</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="13" t="n">
         <v>2807.79</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="13" t="n">
         <v>1993.01</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="13" t="n">
         <v>1654.54</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="13" t="n">
         <v>4759.51</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="13" t="n">
         <v>3113.93</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="13" t="n">
         <v>2174.46</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="13" t="n">
         <v>1869.38</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
         <v>4788.02</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="13" t="n">
         <v>3146.79</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="13" t="n">
         <v>2187.14</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="13" t="n">
         <v>1959.37</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="13" t="n">
         <v>3839.56</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="13" t="n">
         <v>2696.16</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="13" t="n">
         <v>1873.45</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="13" t="n">
         <v>1775.97</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="13" t="n">
         <v>4103.74</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="13" t="n">
         <v>2738.61</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="13" t="n">
         <v>1859.57</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="13" t="n">
         <v>1679.72</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="13" t="n">
         <v>4756.39</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="13" t="n">
         <v>3356.72</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="13" t="n">
         <v>2302.84</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="13" t="n">
         <v>2048.69</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="13" t="n">
         <v>6058.99</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="13" t="n">
         <v>3884.89</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="13" t="n">
         <v>2601.8</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="13" t="n">
         <v>2309.93</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="13" t="n">
         <v>5277.03</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="13" t="n">
         <v>3369.31</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="13" t="n">
         <v>2232.68</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="13" t="n">
         <v>2063.36</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="13" t="n">
         <v>6233.17</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="13" t="n">
         <v>4065.68</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="13" t="n">
         <v>2692.83</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="13" t="n">
         <v>2299.79</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="13" t="n">
         <v>4752.28</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="13" t="n">
         <v>3342.59</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="13" t="n">
         <v>2267.34</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="13" t="n">
         <v>1961.41</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="13" t="n">
         <v>4747.02</v>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="13" t="n">
         <v>3205.88</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="13" t="n">
         <v>2195.46</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="13" t="n">
         <v>1894.23</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="13" t="n">
         <v>4331.31</v>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="13" t="n">
         <v>3043.06</v>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D21" s="13" t="n">
         <v>2155.33</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="13" t="n">
         <v>1846.76</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="13" t="n">
         <v>4642.41</v>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="13" t="n">
         <v>3224.39</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="13" t="n">
         <v>2286.24</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="13" t="n">
         <v>1967.98</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="13" t="n">
         <v>5155.24</v>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C23" s="13" t="n">
         <v>3480.66</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D23" s="13" t="n">
         <v>2528.93</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="13" t="n">
         <v>2234.2</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="13" t="n">
         <v>5514.56</v>
       </c>
-      <c r="C24" s="11" t="n">
+      <c r="C24" s="13" t="n">
         <v>3547.08</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="13" t="n">
         <v>2640.82</v>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="13" t="n">
         <v>2364.36</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B25" s="13" t="n">
         <v>3970.65</v>
       </c>
-      <c r="C25" s="11" t="n">
+      <c r="C25" s="13" t="n">
         <v>2707.08</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="13" t="n">
         <v>2050.6</v>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="13" t="n">
         <v>1923.85</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="13" t="n">
         <v>4211.24</v>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C26" s="13" t="n">
         <v>2732.12</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="13" t="n">
         <v>2075.93</v>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="13" t="n">
         <v>1937.2</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="13" t="n">
         <v>5838.23</v>
       </c>
-      <c r="C27" s="11" t="n">
+      <c r="C27" s="13" t="n">
         <v>3985.87</v>
       </c>
-      <c r="D27" s="11" t="n">
+      <c r="D27" s="13" t="n">
         <v>2896.45</v>
       </c>
-      <c r="E27" s="11" t="n">
+      <c r="E27" s="13" t="n">
         <v>2603.43</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="13" t="n">
         <v>6932.38</v>
       </c>
-      <c r="C28" s="11" t="n">
+      <c r="C28" s="13" t="n">
         <v>4194.06</v>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D28" s="13" t="n">
         <v>3062.61</v>
       </c>
-      <c r="E28" s="11" t="n">
+      <c r="E28" s="13" t="n">
         <v>2846.29</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B29" s="13" t="n">
         <v>6274.09</v>
       </c>
-      <c r="C29" s="11" t="n">
+      <c r="C29" s="13" t="n">
         <v>3775.58</v>
       </c>
-      <c r="D29" s="11" t="n">
+      <c r="D29" s="13" t="n">
         <v>2743.97</v>
       </c>
-      <c r="E29" s="11" t="n">
+      <c r="E29" s="13" t="n">
         <v>2602.94</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="13" t="n">
         <v>5657.15</v>
       </c>
-      <c r="C30" s="11" t="n">
+      <c r="C30" s="13" t="n">
         <v>3718.79</v>
       </c>
-      <c r="D30" s="11" t="n">
+      <c r="D30" s="13" t="n">
         <v>2654.53</v>
       </c>
-      <c r="E30" s="11" t="n">
+      <c r="E30" s="13" t="n">
         <v>2521.24</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n">
+      <c r="B31" s="13" t="n">
         <v>4351.17</v>
       </c>
-      <c r="C31" s="11" t="n">
+      <c r="C31" s="13" t="n">
         <v>2998.46</v>
       </c>
-      <c r="D31" s="11" t="n">
+      <c r="D31" s="13" t="n">
         <v>2171.42</v>
       </c>
-      <c r="E31" s="11" t="n">
+      <c r="E31" s="13" t="n">
         <v>2082.18</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="13" t="n">
         <v>3927.1</v>
       </c>
-      <c r="C32" s="11" t="n">
+      <c r="C32" s="13" t="n">
         <v>2628.2</v>
       </c>
-      <c r="D32" s="11" t="n">
+      <c r="D32" s="13" t="n">
         <v>2018.32</v>
       </c>
-      <c r="E32" s="11" t="n">
+      <c r="E32" s="13" t="n">
         <v>1832.02</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="13" t="n">
         <v>3645.65</v>
       </c>
-      <c r="C33" s="11" t="n">
+      <c r="C33" s="13" t="n">
         <v>2586.18</v>
       </c>
-      <c r="D33" s="11" t="n">
+      <c r="D33" s="13" t="n">
         <v>1941.86</v>
       </c>
-      <c r="E33" s="11" t="n">
+      <c r="E33" s="13" t="n">
         <v>1810.72</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="13" t="n">
         <v>3558.1</v>
       </c>
-      <c r="C34" s="11" t="n">
+      <c r="C34" s="13" t="n">
         <v>2566.63</v>
       </c>
-      <c r="D34" s="11" t="n">
+      <c r="D34" s="13" t="n">
         <v>1978.07</v>
       </c>
-      <c r="E34" s="11" t="n">
+      <c r="E34" s="13" t="n">
         <v>1805.77</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="13" t="n">
         <v>4369.3</v>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C35" s="13" t="n">
         <v>2818.73</v>
       </c>
-      <c r="D35" s="11" t="n">
+      <c r="D35" s="13" t="n">
         <v>2212.31</v>
       </c>
-      <c r="E35" s="11" t="n">
+      <c r="E35" s="13" t="n">
         <v>2076.59</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
       </c>
-      <c r="B36" s="11" t="n">
+      <c r="B36" s="13" t="n">
         <v>4669.24</v>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C36" s="13" t="n">
         <v>2957</v>
       </c>
-      <c r="D36" s="11" t="n">
+      <c r="D36" s="13" t="n">
         <v>2334.22</v>
       </c>
-      <c r="E36" s="11" t="n">
+      <c r="E36" s="13" t="n">
         <v>2181.62</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B37" s="13" t="n">
         <v>3401.01</v>
       </c>
-      <c r="C37" s="11" t="n">
+      <c r="C37" s="13" t="n">
         <v>2466.51</v>
       </c>
-      <c r="D37" s="11" t="n">
+      <c r="D37" s="13" t="n">
         <v>1952.57</v>
       </c>
-      <c r="E37" s="11" t="n">
+      <c r="E37" s="13" t="n">
         <v>1771.54</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B38" s="11" t="n">
+      <c r="B38" s="13" t="n">
         <v>4376.68</v>
       </c>
-      <c r="C38" s="11" t="n">
+      <c r="C38" s="13" t="n">
         <v>2731.84</v>
       </c>
-      <c r="D38" s="11" t="n">
+      <c r="D38" s="13" t="n">
         <v>2062.97</v>
       </c>
-      <c r="E38" s="11" t="n">
+      <c r="E38" s="13" t="n">
         <v>1952.5</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n">
+      <c r="B39" s="13" t="n">
         <v>5368.75</v>
       </c>
-      <c r="C39" s="11" t="n">
+      <c r="C39" s="13" t="n">
         <v>3525.9</v>
       </c>
-      <c r="D39" s="11" t="n">
+      <c r="D39" s="13" t="n">
         <v>2631.02</v>
       </c>
-      <c r="E39" s="11" t="n">
+      <c r="E39" s="13" t="n">
         <v>2393.99</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B40" s="11" t="n">
+      <c r="B40" s="13" t="n">
         <v>6669.43</v>
       </c>
-      <c r="C40" s="11" t="n">
+      <c r="C40" s="13" t="n">
         <v>3942.16</v>
       </c>
-      <c r="D40" s="11" t="n">
+      <c r="D40" s="13" t="n">
         <v>2893.85</v>
       </c>
-      <c r="E40" s="11" t="n">
+      <c r="E40" s="13" t="n">
         <v>2616.97</v>
       </c>
     </row>

</xml_diff>